<commit_message>
Aggiornamento esiti test 448/449 e checklist post-correzioni CDA
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#HENRYSCHEINONEXX/orisline/orisdent/1/report-checklist.xlsx
+++ b/GATEWAY/A1#111#HENRYSCHEINONEXX/orisline/orisdent/1/report-checklist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.aurilia\Documents\Fse\PR-docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.aurilia\Documents\Fse\PR-docs\Repo\GATEWAY\A1#111#HENRYSCHEINONEXX\orisline\orisdent\1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDAD8D7-4EF5-4DC3-BB1F-55C56C528661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F9E09F-9FC8-4B66-BE04-D88446F8D69D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -932,21 +932,6 @@
     <t>Validazione rifiutata: Gateway FSE 400 (/msg/syntax): ERROR: -1,-1 cvc-enumeration-valid: Value 'KO' is not facet-valid with respect to enumeration '[FLFS, OCCR, OREF, SCH]'. It must be a value from the enumeration.,ERROR: -1,-1 cvc-attribute.3: The value 'KO' of attribute 'typeCode' on element 'inFulfillmentOf' is not valid with respect to its type, 'ActRelationshipFulfills'.</t>
   </si>
   <si>
-    <t>2026-03-17T10:02:54Z</t>
-  </si>
-  <si>
-    <t>86244d638d08a7ed1a3fd4dcb7b851fb</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.471c05df51^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>ae0ab2488a95478b48b102b346b43ed1</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.fcd870b295^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>2026-03-17T10:02:55Z</t>
   </si>
   <si>
@@ -1063,6 +1048,21 @@
   </si>
   <si>
     <t>UNKNOWN_WORKFLOW_ID</t>
+  </si>
+  <si>
+    <t>2026-03-27T16:04:48Z</t>
+  </si>
+  <si>
+    <t>65214ae4805430313c1b8d93eafcde14</t>
+  </si>
+  <si>
+    <t>23492374843d186ceb7b487657d57cf3</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.cf14691f58^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.23bba43df7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -3528,7 +3528,7 @@
         <v>179</v>
       </c>
       <c r="I13" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J13" s="33" t="s">
         <v>59</v>
@@ -3591,7 +3591,7 @@
         <v>181</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J14" s="33" t="s">
         <v>59</v>
@@ -3654,7 +3654,7 @@
         <v>183</v>
       </c>
       <c r="I15" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J15" s="33" t="s">
         <v>59</v>
@@ -3717,7 +3717,7 @@
         <v>188</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J16" s="33" t="s">
         <v>59</v>
@@ -3780,7 +3780,7 @@
         <v>191</v>
       </c>
       <c r="I17" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J17" s="33" t="s">
         <v>59</v>
@@ -3843,7 +3843,7 @@
         <v>194</v>
       </c>
       <c r="I18" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J18" s="33" t="s">
         <v>59</v>
@@ -3906,7 +3906,7 @@
         <v>196</v>
       </c>
       <c r="I19" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J19" s="33" t="s">
         <v>59</v>
@@ -3969,7 +3969,7 @@
         <v>199</v>
       </c>
       <c r="I20" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J20" s="33" t="s">
         <v>59</v>
@@ -4032,7 +4032,7 @@
         <v>202</v>
       </c>
       <c r="I21" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J21" s="33" t="s">
         <v>59</v>
@@ -4095,7 +4095,7 @@
         <v>205</v>
       </c>
       <c r="I22" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J22" s="33" t="s">
         <v>59</v>
@@ -4158,7 +4158,7 @@
         <v>206</v>
       </c>
       <c r="I23" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J23" s="33" t="s">
         <v>59</v>
@@ -4221,7 +4221,7 @@
         <v>209</v>
       </c>
       <c r="I24" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J24" s="33" t="s">
         <v>59</v>
@@ -4284,7 +4284,7 @@
         <v>212</v>
       </c>
       <c r="I25" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J25" s="33" t="s">
         <v>59</v>
@@ -4347,7 +4347,7 @@
         <v>215</v>
       </c>
       <c r="I26" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J26" s="33" t="s">
         <v>59</v>
@@ -4410,7 +4410,7 @@
         <v>218</v>
       </c>
       <c r="I27" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J27" s="33" t="s">
         <v>59</v>
@@ -4447,7 +4447,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="130.19999999999999" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="31">
         <v>448</v>
       </c>
@@ -4464,16 +4464,16 @@
         <v>93</v>
       </c>
       <c r="F28" s="32">
-        <v>46098</v>
+        <v>46108</v>
       </c>
       <c r="G28" s="32" t="s">
-        <v>220</v>
+        <v>255</v>
       </c>
       <c r="H28" s="32" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>222</v>
+        <v>258</v>
       </c>
       <c r="J28" s="33" t="s">
         <v>59</v>
@@ -4496,7 +4496,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="130.19999999999999" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="31">
         <v>449</v>
       </c>
@@ -4513,16 +4513,16 @@
         <v>95</v>
       </c>
       <c r="F29" s="32">
-        <v>46098</v>
+        <v>46108</v>
       </c>
       <c r="G29" s="32" t="s">
-        <v>220</v>
+        <v>255</v>
       </c>
       <c r="H29" s="32" t="s">
-        <v>223</v>
+        <v>257</v>
       </c>
       <c r="I29" s="37" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="J29" s="33" t="s">
         <v>59</v>
@@ -4565,13 +4565,13 @@
         <v>46098</v>
       </c>
       <c r="G30" s="31" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="H30" s="31" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="I30" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J30" s="33" t="s">
         <v>59</v>
@@ -4628,13 +4628,13 @@
         <v>46098</v>
       </c>
       <c r="G31" s="31" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="H31" s="31" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="I31" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J31" s="33" t="s">
         <v>59</v>
@@ -4648,7 +4648,7 @@
         <v>59</v>
       </c>
       <c r="O31" s="31" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="P31" s="33" t="s">
         <v>170</v>
@@ -4691,13 +4691,13 @@
         <v>46098</v>
       </c>
       <c r="G32" s="32" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="H32" s="32" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="I32" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J32" s="33" t="s">
         <v>59</v>
@@ -4711,7 +4711,7 @@
         <v>59</v>
       </c>
       <c r="O32" s="33" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="P32" s="33" t="s">
         <v>170</v>
@@ -4734,7 +4734,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="115.8" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="31">
         <v>479</v>
       </c>
@@ -4754,13 +4754,13 @@
         <v>46099</v>
       </c>
       <c r="G33" s="32" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="H33" s="32" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="I33" s="37" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="J33" s="33" t="s">
         <v>59</v>
@@ -4783,7 +4783,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="115.8" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="31">
         <v>480</v>
       </c>
@@ -4803,13 +4803,13 @@
         <v>46099</v>
       </c>
       <c r="G34" s="32" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="H34" s="32" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="I34" s="37" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="J34" s="33" t="s">
         <v>59</v>
@@ -4852,13 +4852,13 @@
         <v>46099</v>
       </c>
       <c r="G35" s="32" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="H35" s="32" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="I35" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J35" s="33" t="s">
         <v>59</v>
@@ -4915,13 +4915,13 @@
         <v>46099</v>
       </c>
       <c r="G36" s="32" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="H36" s="32" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="I36" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J36" s="33" t="s">
         <v>59</v>
@@ -4935,7 +4935,7 @@
         <v>59</v>
       </c>
       <c r="O36" s="33" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="P36" s="33" t="s">
         <v>170</v>
@@ -4978,13 +4978,13 @@
         <v>46099</v>
       </c>
       <c r="G37" s="32" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="H37" s="32" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="I37" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J37" s="33" t="s">
         <v>59</v>
@@ -4998,7 +4998,7 @@
         <v>59</v>
       </c>
       <c r="O37" s="33" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="P37" s="33" t="s">
         <v>170</v>
@@ -5041,13 +5041,13 @@
         <v>46099</v>
       </c>
       <c r="G38" s="32" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="H38" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="I38" s="37" t="s">
         <v>254</v>
-      </c>
-      <c r="I38" s="37" t="s">
-        <v>259</v>
       </c>
       <c r="J38" s="33" t="s">
         <v>59</v>
@@ -5104,13 +5104,13 @@
         <v>46099</v>
       </c>
       <c r="G39" s="32" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="H39" s="32" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="I39" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J39" s="33" t="s">
         <v>59</v>
@@ -5124,7 +5124,7 @@
         <v>59</v>
       </c>
       <c r="O39" s="33" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="P39" s="33" t="s">
         <v>170</v>
@@ -5167,13 +5167,13 @@
         <v>46099</v>
       </c>
       <c r="G40" s="32" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="H40" s="32" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="I40" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J40" s="33" t="s">
         <v>59</v>
@@ -5187,7 +5187,7 @@
         <v>59</v>
       </c>
       <c r="O40" s="33" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="P40" s="33" t="s">
         <v>170</v>
@@ -5230,13 +5230,13 @@
         <v>46099</v>
       </c>
       <c r="G41" s="32" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="H41" s="32" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="I41" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J41" s="33" t="s">
         <v>59</v>
@@ -5250,7 +5250,7 @@
         <v>59</v>
       </c>
       <c r="O41" s="33" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="P41" s="33" t="s">
         <v>170</v>
@@ -5293,13 +5293,13 @@
         <v>46099</v>
       </c>
       <c r="G42" s="32" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="H42" s="32" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="J42" s="33" t="s">
         <v>59</v>
@@ -8413,11 +8413,6 @@
     <filterColumn colId="9">
       <filters>
         <filter val="SI"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="22">
-      <filters>
-        <filter val="KO"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -10738,6 +10733,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -11001,42 +11017,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11059,9 +11043,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Aggiornamento data.json e checklist test 449
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#HENRYSCHEINONEXX/orisline/orisdent/1/report-checklist.xlsx
+++ b/GATEWAY/A1#111#HENRYSCHEINONEXX/orisline/orisdent/1/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.aurilia\Documents\Fse\PR-docs\Repo\GATEWAY\A1#111#HENRYSCHEINONEXX\orisline\orisdent\1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC53970-9E1B-4151-BD42-388474B673CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2149000-0250-4D9C-B26C-D7C3E1651D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1605" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1053,19 +1053,19 @@
     <t>2026-04-02T09:34:42Z</t>
   </si>
   <si>
-    <t>2026-04-02T09:34:43Z</t>
-  </si>
-  <si>
     <t>5013d55bd8e38d5518bf9eecbcfd3d8f</t>
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.83b1a19b4f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>78e3e50dd35577513ab7edea51911cf9</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.ce4234309f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-08T08:01:32Z</t>
+  </si>
+  <si>
+    <t>ec9a5518a8251c75930be9b934572f7e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.1.4.5.1.261da7a2d2a5ad53ed7aca46fb2a8ce1a39614818ddddfa0dd74adba531c29d8.c50d6d0424^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -4473,10 +4473,10 @@
         <v>255</v>
       </c>
       <c r="H28" s="32" t="s">
+        <v>256</v>
+      </c>
+      <c r="I28" s="37" t="s">
         <v>257</v>
-      </c>
-      <c r="I28" s="37" t="s">
-        <v>258</v>
       </c>
       <c r="J28" s="33" t="s">
         <v>59</v>
@@ -4516,10 +4516,10 @@
         <v>95</v>
       </c>
       <c r="F29" s="32">
-        <v>46114</v>
+        <v>46120</v>
       </c>
       <c r="G29" s="32" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="H29" s="32" t="s">
         <v>259</v>
@@ -10736,6 +10736,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -10999,42 +11020,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11057,9 +11046,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>